<commit_message>
chore: complete Agentic CRAG rename
</commit_message>
<xml_diff>
--- a/documents/06_risk_register_and_incidents.xlsx
+++ b/documents/06_risk_register_and_incidents.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Link insight-ai site, remove default site, validate nginx -t, reload nginx</t>
+          <t>Link agentic-crag site, remove default site, validate nginx -t, reload nginx</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Install/link insight-ai Nginx config and reload service</t>
+          <t>Install/link agentic-crag Nginx config and reload service</t>
         </is>
       </c>
     </row>

</xml_diff>